<commit_message>
Devolver id al modificare informacion del gafete
</commit_message>
<xml_diff>
--- a/ASIGNACIONES_LABORALES.xlsx
+++ b/ASIGNACIONES_LABORALES.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Isidro\Documents\SIRH\SIRH-SCRIP-PLANTILLA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilesm\Documents\scriptJSON\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FD375F3-3AC4-4EC5-A911-3886CB04BE76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65BC977B-DB4C-46DD-8E85-C01888BFEC17}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{BD02FFF9-9AE9-4B9D-B85B-9822812C0452}"/>
   </bookViews>
@@ -1285,7 +1285,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1295,6 +1295,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1328,7 +1336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1338,6 +1346,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1653,36 +1662,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFBEA9C7-4E4F-4765-A1BF-F3EFCD719F27}">
   <dimension ref="A1:C314"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.7265625" customWidth="1"/>
-    <col min="2" max="2" width="44.1796875" customWidth="1"/>
-    <col min="3" max="3" width="37.54296875" customWidth="1"/>
+    <col min="1" max="1" width="51.7109375" customWidth="1"/>
+    <col min="2" max="2" width="44.140625" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1693,7 +1702,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1704,7 +1713,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1715,7 +1724,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1726,7 +1735,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -1737,7 +1746,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1748,7 +1757,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1759,7 +1768,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1770,7 +1779,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1781,7 +1790,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1792,7 +1801,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1803,7 +1812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -1814,7 +1823,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1825,7 +1834,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1836,7 +1845,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1847,7 +1856,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1858,7 +1867,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -1869,7 +1878,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -1880,7 +1889,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -1891,7 +1900,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1902,7 +1911,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1913,7 +1922,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -1924,7 +1933,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>43</v>
       </c>
@@ -1935,7 +1944,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -1946,7 +1955,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -1957,7 +1966,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -1968,7 +1977,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>50</v>
       </c>
@@ -1979,7 +1988,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>52</v>
       </c>
@@ -1990,7 +1999,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>54</v>
       </c>
@@ -2001,7 +2010,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>57</v>
       </c>
@@ -2012,7 +2021,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>52</v>
       </c>
@@ -2023,7 +2032,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>60</v>
       </c>
@@ -2034,7 +2043,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>54</v>
       </c>
@@ -2045,7 +2054,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>63</v>
       </c>
@@ -2056,7 +2065,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>65</v>
       </c>
@@ -2067,7 +2076,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>63</v>
       </c>
@@ -2078,7 +2087,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>52</v>
       </c>
@@ -2089,7 +2098,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>52</v>
       </c>
@@ -2100,7 +2109,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>70</v>
       </c>
@@ -2111,7 +2120,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>72</v>
       </c>
@@ -2122,7 +2131,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>74</v>
       </c>
@@ -2133,7 +2142,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>76</v>
       </c>
@@ -2144,7 +2153,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>76</v>
       </c>
@@ -2155,7 +2164,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>76</v>
       </c>
@@ -2166,7 +2175,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>80</v>
       </c>
@@ -2177,7 +2186,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>82</v>
       </c>
@@ -2188,7 +2197,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>84</v>
       </c>
@@ -2199,7 +2208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>80</v>
       </c>
@@ -2210,7 +2219,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>82</v>
       </c>
@@ -2221,7 +2230,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>82</v>
       </c>
@@ -2232,7 +2241,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>82</v>
       </c>
@@ -2243,7 +2252,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>82</v>
       </c>
@@ -2254,7 +2263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>91</v>
       </c>
@@ -2265,7 +2274,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>93</v>
       </c>
@@ -2276,7 +2285,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>91</v>
       </c>
@@ -2287,7 +2296,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -2298,7 +2307,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>97</v>
       </c>
@@ -2309,7 +2318,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>97</v>
       </c>
@@ -2320,7 +2329,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>93</v>
       </c>
@@ -2331,7 +2340,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>93</v>
       </c>
@@ -2342,7 +2351,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>93</v>
       </c>
@@ -2353,7 +2362,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>93</v>
       </c>
@@ -2364,7 +2373,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>104</v>
       </c>
@@ -2375,7 +2384,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>104</v>
       </c>
@@ -2386,7 +2395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>104</v>
       </c>
@@ -2397,7 +2406,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>104</v>
       </c>
@@ -2408,7 +2417,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>109</v>
       </c>
@@ -2419,7 +2428,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>109</v>
       </c>
@@ -2430,7 +2439,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>109</v>
       </c>
@@ -2441,7 +2450,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>109</v>
       </c>
@@ -2452,7 +2461,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>109</v>
       </c>
@@ -2463,7 +2472,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>115</v>
       </c>
@@ -2474,7 +2483,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>117</v>
       </c>
@@ -2485,7 +2494,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>97</v>
       </c>
@@ -2496,7 +2505,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>93</v>
       </c>
@@ -2507,7 +2516,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>93</v>
       </c>
@@ -2518,7 +2527,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>13</v>
       </c>
@@ -2529,7 +2538,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>7</v>
       </c>
@@ -2540,7 +2549,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>7</v>
       </c>
@@ -2551,7 +2560,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>7</v>
       </c>
@@ -2562,7 +2571,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>7</v>
       </c>
@@ -2573,7 +2582,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>7</v>
       </c>
@@ -2584,7 +2593,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>7</v>
       </c>
@@ -2595,7 +2604,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>7</v>
       </c>
@@ -2606,7 +2615,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>7</v>
       </c>
@@ -2617,7 +2626,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>7</v>
       </c>
@@ -2628,7 +2637,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>7</v>
       </c>
@@ -2639,7 +2648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>7</v>
       </c>
@@ -2650,7 +2659,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>7</v>
       </c>
@@ -2661,7 +2670,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>7</v>
       </c>
@@ -2672,7 +2681,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>7</v>
       </c>
@@ -2683,7 +2692,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>7</v>
       </c>
@@ -2694,7 +2703,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>7</v>
       </c>
@@ -2705,7 +2714,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>7</v>
       </c>
@@ -2716,7 +2725,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>7</v>
       </c>
@@ -2727,7 +2736,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>7</v>
       </c>
@@ -2738,7 +2747,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>7</v>
       </c>
@@ -2749,7 +2758,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>7</v>
       </c>
@@ -2760,7 +2769,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>7</v>
       </c>
@@ -2771,7 +2780,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>7</v>
       </c>
@@ -2782,7 +2791,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>7</v>
       </c>
@@ -2793,7 +2802,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>7</v>
       </c>
@@ -2804,7 +2813,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>7</v>
       </c>
@@ -2815,7 +2824,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>7</v>
       </c>
@@ -2826,7 +2835,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>7</v>
       </c>
@@ -2837,7 +2846,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>7</v>
       </c>
@@ -2848,7 +2857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>7</v>
       </c>
@@ -2859,7 +2868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>7</v>
       </c>
@@ -2870,7 +2879,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>7</v>
       </c>
@@ -2881,7 +2890,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>7</v>
       </c>
@@ -2892,7 +2901,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>7</v>
       </c>
@@ -2903,7 +2912,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>7</v>
       </c>
@@ -2914,7 +2923,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>3</v>
       </c>
@@ -2925,7 +2934,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>3</v>
       </c>
@@ -2936,7 +2945,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>3</v>
       </c>
@@ -2947,7 +2956,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>3</v>
       </c>
@@ -2958,7 +2967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>3</v>
       </c>
@@ -2969,7 +2978,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>3</v>
       </c>
@@ -2980,7 +2989,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>3</v>
       </c>
@@ -2991,7 +3000,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>3</v>
       </c>
@@ -3002,7 +3011,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>3</v>
       </c>
@@ -3013,7 +3022,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>3</v>
       </c>
@@ -3024,7 +3033,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>3</v>
       </c>
@@ -3035,7 +3044,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>3</v>
       </c>
@@ -3046,7 +3055,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>3</v>
       </c>
@@ -3057,7 +3066,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>3</v>
       </c>
@@ -3068,7 +3077,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>3</v>
       </c>
@@ -3079,7 +3088,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>3</v>
       </c>
@@ -3090,7 +3099,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>3</v>
       </c>
@@ -3101,7 +3110,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>3</v>
       </c>
@@ -3112,7 +3121,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>3</v>
       </c>
@@ -3123,7 +3132,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>3</v>
       </c>
@@ -3134,7 +3143,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>3</v>
       </c>
@@ -3145,7 +3154,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>3</v>
       </c>
@@ -3156,7 +3165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>3</v>
       </c>
@@ -3167,7 +3176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>3</v>
       </c>
@@ -3178,7 +3187,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>3</v>
       </c>
@@ -3189,7 +3198,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>3</v>
       </c>
@@ -3200,7 +3209,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>3</v>
       </c>
@@ -3211,7 +3220,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>3</v>
       </c>
@@ -3222,7 +3231,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>187</v>
       </c>
@@ -3233,7 +3242,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>187</v>
       </c>
@@ -3244,7 +3253,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>187</v>
       </c>
@@ -3255,7 +3264,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>187</v>
       </c>
@@ -3266,7 +3275,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>187</v>
       </c>
@@ -3277,7 +3286,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>187</v>
       </c>
@@ -3288,7 +3297,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>187</v>
       </c>
@@ -3299,7 +3308,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>187</v>
       </c>
@@ -3310,7 +3319,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>187</v>
       </c>
@@ -3321,7 +3330,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>9</v>
       </c>
@@ -3332,7 +3341,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>9</v>
       </c>
@@ -3343,7 +3352,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>9</v>
       </c>
@@ -3354,7 +3363,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>9</v>
       </c>
@@ -3365,7 +3374,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>9</v>
       </c>
@@ -3376,7 +3385,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>9</v>
       </c>
@@ -3387,7 +3396,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>9</v>
       </c>
@@ -3398,7 +3407,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>9</v>
       </c>
@@ -3409,7 +3418,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>9</v>
       </c>
@@ -3420,7 +3429,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>9</v>
       </c>
@@ -3431,7 +3440,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>9</v>
       </c>
@@ -3442,7 +3451,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>9</v>
       </c>
@@ -3453,7 +3462,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>9</v>
       </c>
@@ -3464,7 +3473,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>9</v>
       </c>
@@ -3475,7 +3484,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>9</v>
       </c>
@@ -3486,7 +3495,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>9</v>
       </c>
@@ -3497,7 +3506,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>9</v>
       </c>
@@ -3508,7 +3517,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>215</v>
       </c>
@@ -3519,7 +3528,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>215</v>
       </c>
@@ -3530,7 +3539,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>160</v>
       </c>
@@ -3541,7 +3550,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>160</v>
       </c>
@@ -3552,7 +3561,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
         <v>413</v>
       </c>
@@ -3563,7 +3572,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" s="4" t="s">
         <v>47</v>
       </c>
@@ -3574,7 +3583,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" s="4" t="s">
         <v>47</v>
       </c>
@@ -3585,7 +3594,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" s="4" t="s">
         <v>47</v>
       </c>
@@ -3596,7 +3605,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="4" t="s">
         <v>47</v>
       </c>
@@ -3607,7 +3616,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="4" t="s">
         <v>47</v>
       </c>
@@ -3618,7 +3627,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="4" t="s">
         <v>47</v>
       </c>
@@ -3629,7 +3638,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="4" t="s">
         <v>47</v>
       </c>
@@ -3640,7 +3649,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="4" t="s">
         <v>47</v>
       </c>
@@ -3651,7 +3660,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="4" t="s">
         <v>47</v>
       </c>
@@ -3662,7 +3671,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="4" t="s">
         <v>47</v>
       </c>
@@ -3673,7 +3682,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="4" t="s">
         <v>47</v>
       </c>
@@ -3684,7 +3693,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="4" t="s">
         <v>47</v>
       </c>
@@ -3695,7 +3704,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="4" t="s">
         <v>47</v>
       </c>
@@ -3706,7 +3715,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="4" t="s">
         <v>47</v>
       </c>
@@ -3717,7 +3726,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="4" t="s">
         <v>47</v>
       </c>
@@ -3728,7 +3737,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="4" t="s">
         <v>243</v>
       </c>
@@ -3739,7 +3748,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="4" t="s">
         <v>243</v>
       </c>
@@ -3750,7 +3759,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="4" t="s">
         <v>243</v>
       </c>
@@ -3761,7 +3770,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="4" t="s">
         <v>243</v>
       </c>
@@ -3772,7 +3781,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="4" t="s">
         <v>243</v>
       </c>
@@ -3783,7 +3792,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>248</v>
       </c>
@@ -3794,7 +3803,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>248</v>
       </c>
@@ -3805,7 +3814,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>251</v>
       </c>
@@ -3816,7 +3825,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>253</v>
       </c>
@@ -3827,7 +3836,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>255</v>
       </c>
@@ -3838,7 +3847,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>255</v>
       </c>
@@ -3849,7 +3858,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>255</v>
       </c>
@@ -3860,7 +3869,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>259</v>
       </c>
@@ -3871,7 +3880,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="4" t="s">
         <v>243</v>
       </c>
@@ -3882,7 +3891,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>262</v>
       </c>
@@ -3893,7 +3902,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="4" t="s">
         <v>243</v>
       </c>
@@ -3904,7 +3913,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>144</v>
       </c>
@@ -3915,7 +3924,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>144</v>
       </c>
@@ -3926,7 +3935,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>144</v>
       </c>
@@ -3937,7 +3946,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>144</v>
       </c>
@@ -3948,7 +3957,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>144</v>
       </c>
@@ -3959,7 +3968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>144</v>
       </c>
@@ -3970,7 +3979,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>144</v>
       </c>
@@ -3981,7 +3990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>144</v>
       </c>
@@ -3992,7 +4001,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>144</v>
       </c>
@@ -4003,7 +4012,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>144</v>
       </c>
@@ -4014,7 +4023,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>144</v>
       </c>
@@ -4025,7 +4034,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>144</v>
       </c>
@@ -4036,7 +4045,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>144</v>
       </c>
@@ -4047,7 +4056,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>144</v>
       </c>
@@ -4058,7 +4067,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>144</v>
       </c>
@@ -4069,7 +4078,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>144</v>
       </c>
@@ -4080,7 +4089,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>144</v>
       </c>
@@ -4091,7 +4100,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>144</v>
       </c>
@@ -4102,7 +4111,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>5</v>
       </c>
@@ -4113,7 +4122,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>5</v>
       </c>
@@ -4124,7 +4133,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>5</v>
       </c>
@@ -4135,7 +4144,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" s="3" t="s">
         <v>298</v>
       </c>
@@ -4146,7 +4155,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" s="3" t="s">
         <v>289</v>
       </c>
@@ -4157,7 +4166,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" s="3" t="s">
         <v>299</v>
       </c>
@@ -4168,7 +4177,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="3" t="s">
         <v>300</v>
       </c>
@@ -4179,7 +4188,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" s="3" t="s">
         <v>300</v>
       </c>
@@ -4190,7 +4199,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" s="3" t="s">
         <v>300</v>
       </c>
@@ -4201,7 +4210,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" s="3" t="s">
         <v>300</v>
       </c>
@@ -4212,7 +4221,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" s="3" t="s">
         <v>300</v>
       </c>
@@ -4223,7 +4232,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="3" t="s">
         <v>301</v>
       </c>
@@ -4234,7 +4243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" s="3" t="s">
         <v>302</v>
       </c>
@@ -4245,7 +4254,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" s="3" t="s">
         <v>301</v>
       </c>
@@ -4256,7 +4265,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" s="3" t="s">
         <v>305</v>
       </c>
@@ -4267,7 +4276,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="3" t="s">
         <v>307</v>
       </c>
@@ -4278,7 +4287,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" s="3" t="s">
         <v>298</v>
       </c>
@@ -4289,7 +4298,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" s="3" t="s">
         <v>301</v>
       </c>
@@ -4300,7 +4309,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" s="3" t="s">
         <v>301</v>
       </c>
@@ -4311,7 +4320,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" s="3" t="s">
         <v>312</v>
       </c>
@@ -4322,7 +4331,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" s="3" t="s">
         <v>312</v>
       </c>
@@ -4333,7 +4342,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" s="3" t="s">
         <v>312</v>
       </c>
@@ -4344,7 +4353,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="3" t="s">
         <v>312</v>
       </c>
@@ -4355,7 +4364,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" s="3" t="s">
         <v>312</v>
       </c>
@@ -4366,7 +4375,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" s="3" t="s">
         <v>312</v>
       </c>
@@ -4377,7 +4386,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" s="3" t="s">
         <v>312</v>
       </c>
@@ -4388,7 +4397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" s="3" t="s">
         <v>312</v>
       </c>
@@ -4399,7 +4408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" s="3" t="s">
         <v>312</v>
       </c>
@@ -4410,7 +4419,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" s="3" t="s">
         <v>312</v>
       </c>
@@ -4421,7 +4430,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" s="3" t="s">
         <v>312</v>
       </c>
@@ -4432,7 +4441,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" s="3" t="s">
         <v>312</v>
       </c>
@@ -4443,7 +4452,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" s="3" t="s">
         <v>312</v>
       </c>
@@ -4454,7 +4463,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
         <v>312</v>
       </c>
@@ -4465,7 +4474,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" s="3" t="s">
         <v>312</v>
       </c>
@@ -4476,7 +4485,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" s="3" t="s">
         <v>312</v>
       </c>
@@ -4487,7 +4496,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" s="3" t="s">
         <v>312</v>
       </c>
@@ -4498,7 +4507,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" s="3" t="s">
         <v>312</v>
       </c>
@@ -4509,7 +4518,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" s="3" t="s">
         <v>312</v>
       </c>
@@ -4520,7 +4529,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" s="3" t="s">
         <v>312</v>
       </c>
@@ -4531,7 +4540,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" s="3" t="s">
         <v>312</v>
       </c>
@@ -4542,7 +4551,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" s="3" t="s">
         <v>334</v>
       </c>
@@ -4553,7 +4562,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" s="3" t="s">
         <v>334</v>
       </c>
@@ -4564,7 +4573,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" s="3" t="s">
         <v>312</v>
       </c>
@@ -4575,7 +4584,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" s="3" t="s">
         <v>334</v>
       </c>
@@ -4586,7 +4595,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" s="3" t="s">
         <v>334</v>
       </c>
@@ -4597,7 +4606,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" s="3" t="s">
         <v>334</v>
       </c>
@@ -4608,7 +4617,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" s="3" t="s">
         <v>334</v>
       </c>
@@ -4619,7 +4628,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" s="3" t="s">
         <v>334</v>
       </c>
@@ -4630,7 +4639,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" s="3" t="s">
         <v>334</v>
       </c>
@@ -4641,7 +4650,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" s="3" t="s">
         <v>334</v>
       </c>
@@ -4652,7 +4661,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" s="3" t="s">
         <v>334</v>
       </c>
@@ -4663,7 +4672,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" s="3" t="s">
         <v>334</v>
       </c>
@@ -4674,7 +4683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" s="3" t="s">
         <v>350</v>
       </c>
@@ -4685,7 +4694,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" s="3" t="s">
         <v>352</v>
       </c>
@@ -4696,7 +4705,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" s="3" t="s">
         <v>356</v>
       </c>
@@ -4707,7 +4716,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" s="3" t="s">
         <v>357</v>
       </c>
@@ -4718,7 +4727,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" s="3" t="s">
         <v>359</v>
       </c>
@@ -4729,7 +4738,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" s="3" t="s">
         <v>359</v>
       </c>
@@ -4740,7 +4749,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="283" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" s="3" t="s">
         <v>352</v>
       </c>
@@ -4751,7 +4760,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" s="3" t="s">
         <v>352</v>
       </c>
@@ -4762,7 +4771,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="285" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" s="3" t="s">
         <v>352</v>
       </c>
@@ -4773,7 +4782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" s="3" t="s">
         <v>366</v>
       </c>
@@ -4784,7 +4793,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" s="3" t="s">
         <v>368</v>
       </c>
@@ -4795,7 +4804,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288" s="3" t="s">
         <v>288</v>
       </c>
@@ -4806,7 +4815,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289" s="3" t="s">
         <v>288</v>
       </c>
@@ -4817,7 +4826,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290" s="3" t="s">
         <v>373</v>
       </c>
@@ -4828,7 +4837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291" s="3" t="s">
         <v>373</v>
       </c>
@@ -4839,7 +4848,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292" s="3" t="s">
         <v>376</v>
       </c>
@@ -4850,7 +4859,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293" s="3" t="s">
         <v>376</v>
       </c>
@@ -4861,7 +4870,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A294" s="3" t="s">
         <v>376</v>
       </c>
@@ -4872,7 +4881,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295" s="3" t="s">
         <v>376</v>
       </c>
@@ -4883,7 +4892,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296" s="3" t="s">
         <v>383</v>
       </c>
@@ -4894,7 +4903,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="297" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297" s="3" t="s">
         <v>383</v>
       </c>
@@ -4905,7 +4914,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298" s="3" t="s">
         <v>383</v>
       </c>
@@ -4916,7 +4925,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299" s="3" t="s">
         <v>387</v>
       </c>
@@ -4927,7 +4936,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>389</v>
       </c>
@@ -4938,7 +4947,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>389</v>
       </c>
@@ -4949,7 +4958,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>389</v>
       </c>
@@ -4960,7 +4969,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>389</v>
       </c>
@@ -4971,7 +4980,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>389</v>
       </c>
@@ -4982,7 +4991,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>389</v>
       </c>
@@ -4993,7 +5002,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>389</v>
       </c>
@@ -5004,7 +5013,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>389</v>
       </c>
@@ -5015,7 +5024,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>389</v>
       </c>
@@ -5026,7 +5035,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>389</v>
       </c>
@@ -5037,7 +5046,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>389</v>
       </c>
@@ -5048,7 +5057,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>389</v>
       </c>
@@ -5059,7 +5068,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>389</v>
       </c>
@@ -5070,7 +5079,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>404</v>
       </c>
@@ -5081,7 +5090,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>406</v>
       </c>
@@ -5094,5 +5103,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>